<commit_message>
add batteries and gearbox. Some changes in table
</commit_message>
<xml_diff>
--- a/Список комплектующих.xlsx
+++ b/Список комплектующих.xlsx
@@ -8,35 +8,24 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\Root\Desktop\Projects\Github\Inventor\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="8_{73EF3884-63C9-4C7B-A8AA-F87ECE5C74EA}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{F7478276-5227-4A6F-BA69-CC983C5D415E}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15990" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Лист1" sheetId="1" r:id="rId1"/>
   </sheets>
-  <calcPr calcId="191029"/>
+  <calcPr calcId="181029"/>
   <extLst>
     <ext xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" uri="{140A7094-0E35-4892-8432-C4D2E57EDEB5}">
       <x15:workbookPr chartTrackingRefBase="1"/>
-    </ext>
-    <ext xmlns:xcalcf="http://schemas.microsoft.com/office/spreadsheetml/2018/calcfeatures" uri="{B58B0392-4F1F-4190-BB64-5DF3571DCE5F}">
-      <xcalcf:calcFeatures>
-        <xcalcf:feature name="microsoft.com:RD"/>
-        <xcalcf:feature name="microsoft.com:Single"/>
-        <xcalcf:feature name="microsoft.com:FV"/>
-        <xcalcf:feature name="microsoft.com:CNMTM"/>
-        <xcalcf:feature name="microsoft.com:LET_WF"/>
-        <xcalcf:feature name="microsoft.com:LAMBDA_WF"/>
-        <xcalcf:feature name="microsoft.com:ARRAYTEXT_WF"/>
-      </xcalcf:calcFeatures>
     </ext>
   </extLst>
 </workbook>
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="23" uniqueCount="20">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="33" uniqueCount="28">
   <si>
     <t>Редуктор</t>
   </si>
@@ -47,9 +36,6 @@
     <t>Колесо</t>
   </si>
   <si>
-    <t>АКБ</t>
-  </si>
-  <si>
     <t>Название</t>
   </si>
   <si>
@@ -96,6 +82,33 @@
   </si>
   <si>
     <t>FlySky Noble NB4 Pro+</t>
+  </si>
+  <si>
+    <t>АКБ на спиннер</t>
+  </si>
+  <si>
+    <t>АКБ на колеса</t>
+  </si>
+  <si>
+    <t>CNHL Racing Series 9500mAh 29.6V 8S 90C Lipo Battery with QS8 Plug</t>
+  </si>
+  <si>
+    <t>вес итог</t>
+  </si>
+  <si>
+    <t>цена итог</t>
+  </si>
+  <si>
+    <t>CNHL Racing Series 9500mAh 22.2V 6S 90C Lipo Battery with QS8 Plug</t>
+  </si>
+  <si>
+    <t>Примечание</t>
+  </si>
+  <si>
+    <t>Ставим 2 в робота (пока)</t>
+  </si>
+  <si>
+    <t>Ставим 1 в робота (пока)</t>
   </si>
 </sst>
 </file>
@@ -103,7 +116,7 @@
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
   <numFmts count="1">
-    <numFmt numFmtId="166" formatCode="0.000"/>
+    <numFmt numFmtId="164" formatCode="0.000"/>
   </numFmts>
   <fonts count="2" x14ac:knownFonts="1">
     <font>
@@ -143,7 +156,7 @@
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
   </cellStyleXfs>
-  <cellXfs count="4">
+  <cellXfs count="5">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
       <alignment horizontal="center"/>
@@ -151,8 +164,11 @@
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
-    <xf numFmtId="166" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyAlignment="1">
+    <xf numFmtId="164" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyAlignment="1">
       <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
     </xf>
   </cellXfs>
   <cellStyles count="2">
@@ -435,48 +451,52 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
-  <dimension ref="A1:H10"/>
+  <dimension ref="A1:I15"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="1" max="1" width="37.42578125" style="1" customWidth="1"/>
-    <col min="2" max="2" width="37.7109375" style="1" customWidth="1"/>
+    <col min="2" max="2" width="67.42578125" style="1" customWidth="1"/>
     <col min="3" max="3" width="18.28515625" style="1" customWidth="1"/>
     <col min="4" max="4" width="18.140625" customWidth="1"/>
     <col min="5" max="5" width="18" style="1" customWidth="1"/>
     <col min="6" max="6" width="18.140625" style="1" customWidth="1"/>
     <col min="7" max="7" width="18.7109375" style="1" customWidth="1"/>
     <col min="8" max="8" width="14.140625" style="1" customWidth="1"/>
+    <col min="9" max="9" width="25.5703125" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:8" x14ac:dyDescent="0.25">
+    <row r="1" spans="1:9" x14ac:dyDescent="0.25">
       <c r="B1" s="1" t="s">
+        <v>3</v>
+      </c>
+      <c r="C1" s="1" t="s">
         <v>4</v>
       </c>
-      <c r="C1" s="1" t="s">
+      <c r="D1" s="1" t="s">
         <v>5</v>
       </c>
-      <c r="D1" s="1" t="s">
+      <c r="E1" s="1" t="s">
+        <v>14</v>
+      </c>
+      <c r="F1" s="1" t="s">
+        <v>13</v>
+      </c>
+      <c r="G1" s="1" t="s">
+        <v>7</v>
+      </c>
+      <c r="H1" s="1" t="s">
         <v>6</v>
       </c>
-      <c r="E1" s="1" t="s">
-        <v>15</v>
-      </c>
-      <c r="F1" s="1" t="s">
-        <v>14</v>
-      </c>
-      <c r="G1" s="1" t="s">
-        <v>8</v>
-      </c>
-      <c r="H1" s="1" t="s">
-        <v>7</v>
-      </c>
-    </row>
-    <row r="2" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="I1" s="1" t="s">
+        <v>25</v>
+      </c>
+    </row>
+    <row r="2" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A2" s="1" t="s">
+        <v>11</v>
+      </c>
+      <c r="B2" s="1" t="s">
         <v>12</v>
-      </c>
-      <c r="B2" s="1" t="s">
-        <v>13</v>
       </c>
       <c r="C2" s="1">
         <v>4</v>
@@ -496,15 +516,16 @@
         <v>168000</v>
       </c>
       <c r="H2" s="2" t="s">
-        <v>17</v>
-      </c>
-    </row>
-    <row r="3" spans="1:8" x14ac:dyDescent="0.25">
+        <v>16</v>
+      </c>
+      <c r="I2" s="4"/>
+    </row>
+    <row r="3" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A3" s="1" t="s">
-        <v>11</v>
+        <v>10</v>
       </c>
       <c r="B3" s="1" t="s">
-        <v>16</v>
+        <v>15</v>
       </c>
       <c r="C3" s="1">
         <v>2</v>
@@ -516,7 +537,7 @@
         <v>2800</v>
       </c>
       <c r="F3" s="3">
-        <f t="shared" ref="F3:F9" si="1">C3*E3/1000</f>
+        <f t="shared" ref="F3:F10" si="1">C3*E3/1000</f>
         <v>5.6</v>
       </c>
       <c r="G3" s="1">
@@ -524,40 +545,75 @@
         <v>127000</v>
       </c>
       <c r="H3" s="2" t="s">
-        <v>17</v>
-      </c>
-    </row>
-    <row r="4" spans="1:8" x14ac:dyDescent="0.25">
+        <v>16</v>
+      </c>
+      <c r="I3" s="4"/>
+    </row>
+    <row r="4" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A4" s="1" t="s">
+        <v>20</v>
+      </c>
+      <c r="B4" s="1" t="s">
+        <v>24</v>
+      </c>
+      <c r="C4" s="1">
+        <v>6</v>
+      </c>
+      <c r="D4" s="1">
+        <v>11000</v>
+      </c>
+      <c r="E4" s="1">
+        <v>1150</v>
+      </c>
+      <c r="F4" s="1">
+        <f>2*E4/1000</f>
+        <v>2.2999999999999998</v>
+      </c>
+      <c r="G4" s="1">
+        <f t="shared" ref="G4" si="2">D4*C4</f>
+        <v>66000</v>
+      </c>
+      <c r="H4" s="2" t="s">
+        <v>16</v>
+      </c>
+      <c r="I4" s="4" t="s">
+        <v>26</v>
+      </c>
+    </row>
+    <row r="5" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="A5" s="1" t="s">
+        <v>19</v>
+      </c>
+      <c r="B5" s="1" t="s">
+        <v>21</v>
+      </c>
+      <c r="C5" s="1">
         <v>3</v>
       </c>
-      <c r="D4" s="1"/>
-      <c r="F4" s="1">
-        <f t="shared" si="1"/>
-        <v>0</v>
-      </c>
-      <c r="G4" s="1">
-        <f t="shared" ref="G4:G8" si="2">D4*C4</f>
-        <v>0</v>
-      </c>
-    </row>
-    <row r="5" spans="1:8" x14ac:dyDescent="0.25">
-      <c r="A5" s="1" t="s">
-        <v>0</v>
-      </c>
-      <c r="D5" s="1"/>
+      <c r="D5" s="1">
+        <v>20000</v>
+      </c>
+      <c r="E5" s="1">
+        <v>1450</v>
+      </c>
       <c r="F5" s="1">
-        <f t="shared" si="1"/>
-        <v>0</v>
+        <f>E5*1/1000</f>
+        <v>1.45</v>
       </c>
       <c r="G5" s="1">
-        <f t="shared" si="2"/>
-        <v>0</v>
-      </c>
-    </row>
-    <row r="6" spans="1:8" x14ac:dyDescent="0.25">
+        <f t="shared" ref="G5:G9" si="3">D5*C5</f>
+        <v>60000</v>
+      </c>
+      <c r="H5" s="2" t="s">
+        <v>16</v>
+      </c>
+      <c r="I5" s="4" t="s">
+        <v>27</v>
+      </c>
+    </row>
+    <row r="6" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A6" s="1" t="s">
-        <v>2</v>
+        <v>0</v>
       </c>
       <c r="D6" s="1"/>
       <c r="F6" s="1">
@@ -565,13 +621,14 @@
         <v>0</v>
       </c>
       <c r="G6" s="1">
-        <f t="shared" si="2"/>
-        <v>0</v>
-      </c>
-    </row>
-    <row r="7" spans="1:8" x14ac:dyDescent="0.25">
+        <f t="shared" si="3"/>
+        <v>0</v>
+      </c>
+      <c r="I6" s="4"/>
+    </row>
+    <row r="7" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A7" s="1" t="s">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="D7" s="1"/>
       <c r="F7" s="1">
@@ -579,50 +636,38 @@
         <v>0</v>
       </c>
       <c r="G7" s="1">
-        <f t="shared" si="2"/>
-        <v>0</v>
-      </c>
-    </row>
-    <row r="8" spans="1:8" x14ac:dyDescent="0.25">
+        <f t="shared" si="3"/>
+        <v>0</v>
+      </c>
+      <c r="I7" s="4"/>
+    </row>
+    <row r="8" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A8" s="1" t="s">
-        <v>9</v>
-      </c>
-      <c r="B8" s="1" t="s">
-        <v>18</v>
-      </c>
-      <c r="C8" s="1">
         <v>1</v>
       </c>
-      <c r="D8" s="1">
-        <v>30000</v>
-      </c>
-      <c r="E8" s="1">
-        <v>0</v>
-      </c>
+      <c r="D8" s="1"/>
       <c r="F8" s="1">
         <f t="shared" si="1"/>
         <v>0</v>
       </c>
       <c r="G8" s="1">
-        <f t="shared" si="2"/>
-        <v>30000</v>
-      </c>
-      <c r="H8" s="2" t="s">
+        <f t="shared" si="3"/>
+        <v>0</v>
+      </c>
+      <c r="I8" s="4"/>
+    </row>
+    <row r="9" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="A9" s="1" t="s">
+        <v>8</v>
+      </c>
+      <c r="B9" s="1" t="s">
         <v>17</v>
-      </c>
-    </row>
-    <row r="9" spans="1:8" x14ac:dyDescent="0.25">
-      <c r="A9" s="1" t="s">
-        <v>10</v>
-      </c>
-      <c r="B9" s="1" t="s">
-        <v>19</v>
       </c>
       <c r="C9" s="1">
         <v>1</v>
       </c>
       <c r="D9" s="1">
-        <v>54000</v>
+        <v>30000</v>
       </c>
       <c r="E9" s="1">
         <v>0</v>
@@ -632,23 +677,74 @@
         <v>0</v>
       </c>
       <c r="G9" s="1">
-        <f t="shared" ref="G9" si="3">D9*C9</f>
+        <f t="shared" si="3"/>
+        <v>30000</v>
+      </c>
+      <c r="H9" s="2" t="s">
+        <v>16</v>
+      </c>
+      <c r="I9" s="4"/>
+    </row>
+    <row r="10" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="A10" s="1" t="s">
+        <v>9</v>
+      </c>
+      <c r="B10" s="1" t="s">
+        <v>18</v>
+      </c>
+      <c r="C10" s="1">
+        <v>1</v>
+      </c>
+      <c r="D10" s="1">
         <v>54000</v>
       </c>
-      <c r="H9" s="2" t="s">
-        <v>17</v>
-      </c>
-    </row>
-    <row r="10" spans="1:8" x14ac:dyDescent="0.25">
-      <c r="D10" s="1"/>
+      <c r="E10" s="1">
+        <v>0</v>
+      </c>
+      <c r="F10" s="1">
+        <f t="shared" si="1"/>
+        <v>0</v>
+      </c>
+      <c r="G10" s="1">
+        <f t="shared" ref="G10" si="4">D10*C10</f>
+        <v>54000</v>
+      </c>
+      <c r="H10" s="2" t="s">
+        <v>16</v>
+      </c>
+      <c r="I10" s="4"/>
+    </row>
+    <row r="11" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="D11" s="1"/>
+    </row>
+    <row r="14" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="F14" s="1" t="s">
+        <v>22</v>
+      </c>
+      <c r="G14" s="1" t="s">
+        <v>23</v>
+      </c>
+    </row>
+    <row r="15" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="F15" s="3">
+        <f>SUM(F2:F10)</f>
+        <v>16.349999999999998</v>
+      </c>
+      <c r="G15" s="1">
+        <f>SUM(G2:G10)</f>
+        <v>505000</v>
+      </c>
     </row>
   </sheetData>
   <hyperlinks>
     <hyperlink ref="H2" r:id="rId1" xr:uid="{ED112093-5EE6-4CF2-83CB-B26017BF5998}"/>
     <hyperlink ref="H3" r:id="rId2" xr:uid="{4556990F-7CC9-424D-BDCC-CFB4A8311E70}"/>
-    <hyperlink ref="H8" r:id="rId3" xr:uid="{B9BDD22B-89D5-4A04-907B-F4B97FC79D3A}"/>
-    <hyperlink ref="H9" r:id="rId4" xr:uid="{0D367BC3-86AF-49E2-9E5B-0218D76B8696}"/>
+    <hyperlink ref="H9" r:id="rId3" xr:uid="{B9BDD22B-89D5-4A04-907B-F4B97FC79D3A}"/>
+    <hyperlink ref="H10" r:id="rId4" xr:uid="{0D367BC3-86AF-49E2-9E5B-0218D76B8696}"/>
+    <hyperlink ref="H5" r:id="rId5" xr:uid="{E5740DB7-F485-47D6-A269-3A5822239E74}"/>
+    <hyperlink ref="H4" r:id="rId6" xr:uid="{B0163109-7863-4E12-937C-00318DE0FA92}"/>
   </hyperlinks>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+  <pageSetup paperSize="9" orientation="portrait" horizontalDpi="1200" verticalDpi="1200" r:id="rId7"/>
 </worksheet>
 </file>
</xml_diff>

<commit_message>
Moving project to Compas3d
</commit_message>
<xml_diff>
--- a/Список комплектующих.xlsx
+++ b/Список комплектующих.xlsx
@@ -1,24 +1,35 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="6" rupBuild="28623"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="6" rupBuild="27932"/>
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\Root\Desktop\Projects\Github\Inventor\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\tishk\Desktop\Projects\Битва роботов\BOBR\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{F7478276-5227-4A6F-BA69-CC983C5D415E}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{0682AE81-16B8-4689-9181-3339E6E9DAF9}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15990" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-100" yWindow="-100" windowWidth="21467" windowHeight="11443" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Лист1" sheetId="1" r:id="rId1"/>
   </sheets>
-  <calcPr calcId="181029"/>
+  <calcPr calcId="191029"/>
   <extLst>
     <ext xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" uri="{140A7094-0E35-4892-8432-C4D2E57EDEB5}">
       <x15:workbookPr chartTrackingRefBase="1"/>
+    </ext>
+    <ext xmlns:xcalcf="http://schemas.microsoft.com/office/spreadsheetml/2018/calcfeatures" uri="{B58B0392-4F1F-4190-BB64-5DF3571DCE5F}">
+      <xcalcf:calcFeatures>
+        <xcalcf:feature name="microsoft.com:RD"/>
+        <xcalcf:feature name="microsoft.com:Single"/>
+        <xcalcf:feature name="microsoft.com:FV"/>
+        <xcalcf:feature name="microsoft.com:CNMTM"/>
+        <xcalcf:feature name="microsoft.com:LET_WF"/>
+        <xcalcf:feature name="microsoft.com:LAMBDA_WF"/>
+        <xcalcf:feature name="microsoft.com:ARRAYTEXT_WF"/>
+      </xcalcf:calcFeatures>
     </ext>
   </extLst>
 </workbook>
@@ -452,20 +463,20 @@
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
   <dimension ref="A1:I15"/>
-  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
+  <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <cols>
-    <col min="1" max="1" width="37.42578125" style="1" customWidth="1"/>
-    <col min="2" max="2" width="67.42578125" style="1" customWidth="1"/>
-    <col min="3" max="3" width="18.28515625" style="1" customWidth="1"/>
-    <col min="4" max="4" width="18.140625" customWidth="1"/>
+    <col min="1" max="1" width="37.3984375" style="1" customWidth="1"/>
+    <col min="2" max="2" width="67.3984375" style="1" customWidth="1"/>
+    <col min="3" max="3" width="18.296875" style="1" customWidth="1"/>
+    <col min="4" max="4" width="18.09765625" customWidth="1"/>
     <col min="5" max="5" width="18" style="1" customWidth="1"/>
-    <col min="6" max="6" width="18.140625" style="1" customWidth="1"/>
-    <col min="7" max="7" width="18.7109375" style="1" customWidth="1"/>
-    <col min="8" max="8" width="14.140625" style="1" customWidth="1"/>
-    <col min="9" max="9" width="25.5703125" customWidth="1"/>
+    <col min="6" max="6" width="18.09765625" style="1" customWidth="1"/>
+    <col min="7" max="7" width="18.69921875" style="1" customWidth="1"/>
+    <col min="8" max="8" width="14.09765625" style="1" customWidth="1"/>
+    <col min="9" max="9" width="25.59765625" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:9" x14ac:dyDescent="0.25">
+    <row r="1" spans="1:9" x14ac:dyDescent="0.3">
       <c r="B1" s="1" t="s">
         <v>3</v>
       </c>
@@ -491,7 +502,7 @@
         <v>25</v>
       </c>
     </row>
-    <row r="2" spans="1:9" x14ac:dyDescent="0.25">
+    <row r="2" spans="1:9" x14ac:dyDescent="0.3">
       <c r="A2" s="1" t="s">
         <v>11</v>
       </c>
@@ -520,7 +531,7 @@
       </c>
       <c r="I2" s="4"/>
     </row>
-    <row r="3" spans="1:9" x14ac:dyDescent="0.25">
+    <row r="3" spans="1:9" x14ac:dyDescent="0.3">
       <c r="A3" s="1" t="s">
         <v>10</v>
       </c>
@@ -549,7 +560,7 @@
       </c>
       <c r="I3" s="4"/>
     </row>
-    <row r="4" spans="1:9" x14ac:dyDescent="0.25">
+    <row r="4" spans="1:9" x14ac:dyDescent="0.3">
       <c r="A4" s="1" t="s">
         <v>20</v>
       </c>
@@ -580,7 +591,7 @@
         <v>26</v>
       </c>
     </row>
-    <row r="5" spans="1:9" x14ac:dyDescent="0.25">
+    <row r="5" spans="1:9" x14ac:dyDescent="0.3">
       <c r="A5" s="1" t="s">
         <v>19</v>
       </c>
@@ -611,14 +622,20 @@
         <v>27</v>
       </c>
     </row>
-    <row r="6" spans="1:9" x14ac:dyDescent="0.25">
+    <row r="6" spans="1:9" x14ac:dyDescent="0.3">
       <c r="A6" s="1" t="s">
         <v>0</v>
       </c>
+      <c r="C6" s="1">
+        <v>4</v>
+      </c>
       <c r="D6" s="1"/>
+      <c r="E6" s="1">
+        <v>2000</v>
+      </c>
       <c r="F6" s="1">
         <f t="shared" si="1"/>
-        <v>0</v>
+        <v>8</v>
       </c>
       <c r="G6" s="1">
         <f t="shared" si="3"/>
@@ -626,14 +643,20 @@
       </c>
       <c r="I6" s="4"/>
     </row>
-    <row r="7" spans="1:9" x14ac:dyDescent="0.25">
+    <row r="7" spans="1:9" x14ac:dyDescent="0.3">
       <c r="A7" s="1" t="s">
         <v>2</v>
       </c>
+      <c r="C7" s="1">
+        <v>4</v>
+      </c>
       <c r="D7" s="1"/>
+      <c r="E7" s="1">
+        <v>1500</v>
+      </c>
       <c r="F7" s="1">
         <f t="shared" si="1"/>
-        <v>0</v>
+        <v>6</v>
       </c>
       <c r="G7" s="1">
         <f t="shared" si="3"/>
@@ -641,7 +664,7 @@
       </c>
       <c r="I7" s="4"/>
     </row>
-    <row r="8" spans="1:9" x14ac:dyDescent="0.25">
+    <row r="8" spans="1:9" x14ac:dyDescent="0.3">
       <c r="A8" s="1" t="s">
         <v>1</v>
       </c>
@@ -656,7 +679,7 @@
       </c>
       <c r="I8" s="4"/>
     </row>
-    <row r="9" spans="1:9" x14ac:dyDescent="0.25">
+    <row r="9" spans="1:9" x14ac:dyDescent="0.3">
       <c r="A9" s="1" t="s">
         <v>8</v>
       </c>
@@ -685,7 +708,7 @@
       </c>
       <c r="I9" s="4"/>
     </row>
-    <row r="10" spans="1:9" x14ac:dyDescent="0.25">
+    <row r="10" spans="1:9" x14ac:dyDescent="0.3">
       <c r="A10" s="1" t="s">
         <v>9</v>
       </c>
@@ -714,10 +737,10 @@
       </c>
       <c r="I10" s="4"/>
     </row>
-    <row r="11" spans="1:9" x14ac:dyDescent="0.25">
+    <row r="11" spans="1:9" x14ac:dyDescent="0.3">
       <c r="D11" s="1"/>
     </row>
-    <row r="14" spans="1:9" x14ac:dyDescent="0.25">
+    <row r="14" spans="1:9" x14ac:dyDescent="0.3">
       <c r="F14" s="1" t="s">
         <v>22</v>
       </c>
@@ -725,10 +748,10 @@
         <v>23</v>
       </c>
     </row>
-    <row r="15" spans="1:9" x14ac:dyDescent="0.25">
+    <row r="15" spans="1:9" x14ac:dyDescent="0.3">
       <c r="F15" s="3">
         <f>SUM(F2:F10)</f>
-        <v>16.349999999999998</v>
+        <v>30.349999999999998</v>
       </c>
       <c r="G15" s="1">
         <f>SUM(G2:G10)</f>

</xml_diff>